<commit_message>
feat: connect real icon generation workflow
</commit_message>
<xml_diff>
--- a/outputs/2026-08-22-style-preview-deployment/IconGen-前后端原子级开发计划.xlsx
+++ b/outputs/2026-08-22-style-preview-deployment/IconGen-前后端原子级开发计划.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段概览" sheetId="1" r:id="R527e9c38e14440de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前端开发计划" sheetId="2" r:id="Re800f3869faa48e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后端开发计划" sheetId="3" r:id="R9a58456a17734bee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段概览" sheetId="1" r:id="R6980427b4e9e4a02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前端开发计划" sheetId="2" r:id="Rbca078a026314d46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后端开发计划" sheetId="3" r:id="R52f9f5715f9046f1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -205,7 +205,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FrontendAtomicPlan" displayName="FrontendAtomicPlan" ref="A3:R268" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FrontendAtomicPlan" displayName="FrontendAtomicPlan" ref="A3:R270" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="阶段"/>
     <x:tableColumn id="2" name="大需求/业务模块"/>
@@ -231,7 +231,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BackendAtomicPlan" displayName="BackendAtomicPlan" ref="A3:R277" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BackendAtomicPlan" displayName="BackendAtomicPlan" ref="A3:R278" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="阶段"/>
     <x:tableColumn id="2" name="大需求/业务模块"/>
@@ -475,7 +475,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>更新时间：2026-08-24；完成生成表单组件化重构、交互图标与App图标用途协议贯通；默认图形结构改为线性；简化空主体校验提示；Shared、Web、Worker测试与相关工作区类型检查通过</x:v>
+        <x:v>更新时间：2026-08-25；完成逐项追加图标主体输入、移除输入hint、真实Image 2/Sub2API本地生成链路、结果页实时回显与ZIP下载修复、我的图标接入当前用户Supabase真实任务；Shared、Web、Worker测试与相关类型检查通过</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
@@ -515,17 +515,17 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="D4" s="14" t="n">
-        <x:v>265</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="E4" s="14" t="n">
-        <x:v>147</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="F4" s="14" t="n">
         <x:v>118</x:v>
       </x:c>
       <x:c r="G4" s="15" t="n">
         <x:f>E4/D4</x:f>
-        <x:v>0.5547169811320755</x:v>
+        <x:v>0.5580524344569289</x:v>
       </x:c>
       <x:c r="H4" s="14" t="str">
         <x:v>一个动作、一个交付物、一个独立验收结果</x:v>
@@ -542,17 +542,17 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="D5" s="14" t="n">
-        <x:v>293</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="E5" s="14" t="n">
         <x:v>110</x:v>
       </x:c>
       <x:c r="F5" s="14" t="n">
-        <x:v>183</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="G5" s="15" t="n">
         <x:f>E5/D5</x:f>
-        <x:v>0.37542662116040953</x:v>
+        <x:v>0.3793103448275862</x:v>
       </x:c>
       <x:c r="H5" s="14" t="str">
         <x:v>一个动作、一个交付物、一个独立验收结果</x:v>
@@ -730,7 +730,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O4" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P4" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -786,7 +786,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O5" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P5" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -842,7 +842,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O6" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P6" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -898,7 +898,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O7" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P7" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -954,7 +954,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O8" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P8" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -1010,7 +1010,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O9" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P9" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -1066,7 +1066,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O10" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P10" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -1122,7 +1122,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O11" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P11" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -1178,7 +1178,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O12" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P12" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -1234,7 +1234,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O13" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P13" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -1290,7 +1290,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O14" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P14" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -1346,7 +1346,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O15" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P15" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -1402,7 +1402,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O16" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P16" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -1458,7 +1458,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O17" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P17" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -1514,7 +1514,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O18" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P18" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -1570,7 +1570,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O19" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P19" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -1626,7 +1626,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O20" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P20" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -1682,7 +1682,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O21" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P21" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -14842,7 +14842,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O256" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P256" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -14898,7 +14898,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O257" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P257" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -14954,7 +14954,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O258" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P258" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -15010,7 +15010,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O259" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P259" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -15066,7 +15066,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O260" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P260" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -15524,6 +15524,118 @@
       </x:c>
       <x:c r="R268" t="str">
         <x:v>仅调整默认交互状态与前端提示，不改变存储数据</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269">
+      <x:c r="A269" t="str">
+        <x:v>第 1 期</x:v>
+      </x:c>
+      <x:c r="B269" t="str">
+        <x:v>2. 图片生成与结果</x:v>
+      </x:c>
+      <x:c r="C269" t="str">
+        <x:v>GEN-SUBJECT-001</x:v>
+      </x:c>
+      <x:c r="D269" t="str">
+        <x:v>图标主体输入</x:v>
+      </x:c>
+      <x:c r="E269" t="str">
+        <x:v>FE-GEN-SUBJECT-01</x:v>
+      </x:c>
+      <x:c r="F269" t="str">
+        <x:v>前端</x:v>
+      </x:c>
+      <x:c r="G269" t="str">
+        <x:v>将图标主体改为逐项追加输入</x:v>
+      </x:c>
+      <x:c r="H269" t="str">
+        <x:v>单主体输入列表与追加删除交互</x:v>
+      </x:c>
+      <x:c r="I269" t="str">
+        <x:v>一个输入项严格对应一个图标主体；可追加、删除且最多20项；不再按逗号猜测拆分</x:v>
+      </x:c>
+      <x:c r="J269" t="str">
+        <x:v>FE-GEN-PREVIEW-03</x:v>
+      </x:c>
+      <x:c r="K269" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="L269" t="str">
+        <x:v>08-25</x:v>
+      </x:c>
+      <x:c r="M269" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N269" t="str">
+        <x:v>subjects[]；clientId；MAX_SUBJECTS=20</x:v>
+      </x:c>
+      <x:c r="O269" t="str">
+        <x:v>空白/已填写；1项/多项；可追加/达到上限</x:v>
+      </x:c>
+      <x:c r="P269" t="str">
+        <x:v>空输入提交、删除后索引错位、旧多行解析残留</x:v>
+      </x:c>
+      <x:c r="Q269" t="str">
+        <x:v>icon-subject-editor.tsx；generation-form.tsx；subject-parser.ts；Shared与Web测试、类型检查通过</x:v>
+      </x:c>
+      <x:c r="R269" t="str">
+        <x:v>移除每项placeholder；保留无障碍隐藏标签；每个主体默认3种方案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270">
+      <x:c r="A270" t="str">
+        <x:v>第 1 期</x:v>
+      </x:c>
+      <x:c r="B270" t="str">
+        <x:v>2. 图片生成与结果</x:v>
+      </x:c>
+      <x:c r="C270" t="str">
+        <x:v>GEN-RESULT-001</x:v>
+      </x:c>
+      <x:c r="D270" t="str">
+        <x:v>我的图标与结果回显</x:v>
+      </x:c>
+      <x:c r="E270" t="str">
+        <x:v>FE-GEN-RESULT-01</x:v>
+      </x:c>
+      <x:c r="F270" t="str">
+        <x:v>前端</x:v>
+      </x:c>
+      <x:c r="G270" t="str">
+        <x:v>将我的图标列表切换为真实任务数据</x:v>
+      </x:c>
+      <x:c r="H270" t="str">
+        <x:v>当前用户Supabase生成任务列表</x:v>
+      </x:c>
+      <x:c r="I270" t="str">
+        <x:v>列表不再导入mockJobs；仅查询当前用户任务；排除固定演示任务；按创建时间倒序并可进入真实详情</x:v>
+      </x:c>
+      <x:c r="J270" t="str">
+        <x:v>BE-GEN-RUNTIME-01</x:v>
+      </x:c>
+      <x:c r="K270" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="L270" t="str">
+        <x:v>08-25</x:v>
+      </x:c>
+      <x:c r="M270" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N270" t="str">
+        <x:v>generation_jobs.user_id；generation_subjects.job_id；job_id</x:v>
+      </x:c>
+      <x:c r="O270" t="str">
+        <x:v>无任务/排队中/处理中/已完成/失败</x:v>
+      </x:c>
+      <x:c r="P270" t="str">
+        <x:v>演示任务混入、越权读取、主体为空、数据库查询失败</x:v>
+      </x:c>
+      <x:c r="Q270" t="str">
+        <x:v>generation-job-list-reader.ts；icon-job-list.tsx；/icons服务端页面；Web 15项测试与类型检查通过</x:v>
+      </x:c>
+      <x:c r="R270" t="str">
+        <x:v>详情页、轮询、签名预览URL与ZIP下载均使用真实Supabase数据</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15542,7 +15654,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4fe9dcd13fb4f96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7294616f502c4ca9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15698,7 +15810,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O4" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P4" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -15733,7 +15845,7 @@
         <x:v>建立Worker服务入口</x:v>
       </x:c>
       <x:c r="H5" s="13" t="str">
-        <x:v>SQS handler和依赖装配</x:v>
+        <x:v>生成处理入口和依赖装配</x:v>
       </x:c>
       <x:c r="I5" s="13" t="str">
         <x:v>批次失败按messageId返回</x:v>
@@ -15754,7 +15866,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O5" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P5" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -15810,7 +15922,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O6" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P6" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -15866,7 +15978,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O7" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P7" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -18417,15 +18529,9 @@
       <x:c r="F53" s="13" t="str">
         <x:v>后端</x:v>
       </x:c>
-      <x:c r="G53" s="13" t="str">
-        <x:v>事务提交后投递SQS v2</x:v>
-      </x:c>
-      <x:c r="H53" s="13" t="str">
-        <x:v>jobId/requestedAt消息</x:v>
-      </x:c>
-      <x:c r="I53" s="13" t="str">
-        <x:v>投递失败有补偿/重投策略</x:v>
-      </x:c>
+      <x:c r="G53" s="13"/>
+      <x:c r="H53" s="13"/>
+      <x:c r="I53" s="13"/>
       <x:c r="J53" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
@@ -19257,15 +19363,9 @@
       <x:c r="F68" s="13" t="str">
         <x:v>后端</x:v>
       </x:c>
-      <x:c r="G68" s="13" t="str">
-        <x:v>解析SQS v2消息</x:v>
-      </x:c>
-      <x:c r="H68" s="13" t="str">
-        <x:v>version/jobId/requestedAt</x:v>
-      </x:c>
-      <x:c r="I68" s="13" t="str">
-        <x:v>非法消息进入失败处理</x:v>
-      </x:c>
+      <x:c r="G68" s="13"/>
+      <x:c r="H68" s="13"/>
+      <x:c r="I68" s="13"/>
       <x:c r="J68" s="13" t="str">
         <x:v>—</x:v>
       </x:c>
@@ -30034,7 +30134,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O260" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P260" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -30090,7 +30190,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O261" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P261" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -30103,116 +30203,44 @@
       </x:c>
     </x:row>
     <x:row r="262" ht="68" customHeight="1">
-      <x:c r="A262" s="13" t="str">
-        <x:v>第 3 期</x:v>
-      </x:c>
-      <x:c r="B262" s="13" t="str">
-        <x:v>6. 平台、工程与上线</x:v>
-      </x:c>
-      <x:c r="C262" s="13" t="str">
-        <x:v>INF-001/002</x:v>
-      </x:c>
-      <x:c r="D262" s="13" t="str">
-        <x:v>云部署与可观测性</x:v>
-      </x:c>
-      <x:c r="E262" s="13" t="str">
-        <x:v>BE-DEPLOY-03</x:v>
-      </x:c>
-      <x:c r="F262" s="13" t="str">
-        <x:v>后端</x:v>
-      </x:c>
-      <x:c r="G262" s="13" t="str">
-        <x:v>配置AWS SQS和DLQ</x:v>
-      </x:c>
-      <x:c r="H262" s="13" t="str">
-        <x:v>可见性超时和重试次数</x:v>
-      </x:c>
-      <x:c r="I262" s="13" t="str">
-        <x:v>失败消息进入DLQ</x:v>
-      </x:c>
-      <x:c r="J262" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="K262" s="13" t="str">
-        <x:v>待完成</x:v>
-      </x:c>
-      <x:c r="L262" s="13" t="str">
-        <x:v>09-22～09-24</x:v>
-      </x:c>
-      <x:c r="M262" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="N262" s="13" t="str">
-        <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
-      </x:c>
-      <x:c r="O262" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
-      </x:c>
-      <x:c r="P262" s="13" t="str">
-        <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
-      </x:c>
-      <x:c r="Q262" s="13" t="str">
-        <x:v>环境隔离、最小权限、生产审计、日志脱敏</x:v>
-      </x:c>
-      <x:c r="R262" s="13" t="str">
-        <x:v>部署可回滚；Worker/清理任务可重入；密钥不入库不导出</x:v>
-      </x:c>
+      <x:c r="A262" s="13"/>
+      <x:c r="B262" s="13"/>
+      <x:c r="C262" s="13"/>
+      <x:c r="D262" s="13"/>
+      <x:c r="E262" s="13"/>
+      <x:c r="F262" s="13"/>
+      <x:c r="G262" s="13"/>
+      <x:c r="H262" s="13"/>
+      <x:c r="I262" s="13"/>
+      <x:c r="J262" s="13"/>
+      <x:c r="K262" s="13"/>
+      <x:c r="L262" s="13"/>
+      <x:c r="M262" s="13"/>
+      <x:c r="N262" s="13"/>
+      <x:c r="O262" s="13"/>
+      <x:c r="P262" s="13"/>
+      <x:c r="Q262" s="13"/>
+      <x:c r="R262" s="13"/>
     </x:row>
     <x:row r="263" ht="68" customHeight="1">
-      <x:c r="A263" s="13" t="str">
-        <x:v>第 3 期</x:v>
-      </x:c>
-      <x:c r="B263" s="13" t="str">
-        <x:v>6. 平台、工程与上线</x:v>
-      </x:c>
-      <x:c r="C263" s="13" t="str">
-        <x:v>INF-001/002</x:v>
-      </x:c>
-      <x:c r="D263" s="13" t="str">
-        <x:v>云部署与可观测性</x:v>
-      </x:c>
-      <x:c r="E263" s="13" t="str">
-        <x:v>BE-DEPLOY-04</x:v>
-      </x:c>
-      <x:c r="F263" s="13" t="str">
-        <x:v>后端</x:v>
-      </x:c>
-      <x:c r="G263" s="13" t="str">
-        <x:v>部署Lambda Worker</x:v>
-      </x:c>
-      <x:c r="H263" s="13" t="str">
-        <x:v>内存、超时、并发限制</x:v>
-      </x:c>
-      <x:c r="I263" s="13" t="str">
-        <x:v>单任务成本和超时可控</x:v>
-      </x:c>
-      <x:c r="J263" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="K263" s="13" t="str">
-        <x:v>待完成</x:v>
-      </x:c>
-      <x:c r="L263" s="13" t="str">
-        <x:v>09-22～09-24</x:v>
-      </x:c>
-      <x:c r="M263" s="13" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="N263" s="13" t="str">
-        <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
-      </x:c>
-      <x:c r="O263" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
-      </x:c>
-      <x:c r="P263" s="13" t="str">
-        <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
-      </x:c>
-      <x:c r="Q263" s="13" t="str">
-        <x:v>环境隔离、最小权限、生产审计、日志脱敏</x:v>
-      </x:c>
-      <x:c r="R263" s="13" t="str">
-        <x:v>部署可回滚；Worker/清理任务可重入；密钥不入库不导出</x:v>
-      </x:c>
+      <x:c r="A263" s="13"/>
+      <x:c r="B263" s="13"/>
+      <x:c r="C263" s="13"/>
+      <x:c r="D263" s="13"/>
+      <x:c r="E263" s="13"/>
+      <x:c r="F263" s="13"/>
+      <x:c r="G263" s="13"/>
+      <x:c r="H263" s="13"/>
+      <x:c r="I263" s="13"/>
+      <x:c r="J263" s="13"/>
+      <x:c r="K263" s="13"/>
+      <x:c r="L263" s="13"/>
+      <x:c r="M263" s="13"/>
+      <x:c r="N263" s="13"/>
+      <x:c r="O263" s="13"/>
+      <x:c r="P263" s="13"/>
+      <x:c r="Q263" s="13"/>
+      <x:c r="R263" s="13"/>
     </x:row>
     <x:row r="264" ht="68" customHeight="1">
       <x:c r="A264" s="13" t="str">
@@ -30237,7 +30265,7 @@
         <x:v>配置服务端Secrets</x:v>
       </x:c>
       <x:c r="H264" s="13" t="str">
-        <x:v>OpenAI/Stripe/Supabase/AWS</x:v>
+        <x:v>OpenAI/Stripe/Supabase</x:v>
       </x:c>
       <x:c r="I264" s="13" t="str">
         <x:v>浏览器和仓库无密钥</x:v>
@@ -30258,7 +30286,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O264" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P264" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -30314,7 +30342,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O265" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P265" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -30349,7 +30377,7 @@
         <x:v>建立关键告警</x:v>
       </x:c>
       <x:c r="H266" s="13" t="str">
-        <x:v>DLQ、Webhook失败、余额异常、清理失败</x:v>
+        <x:v>Webhook失败、余额异常、清理失败</x:v>
       </x:c>
       <x:c r="I266" s="13" t="str">
         <x:v>告警包含可定位ID</x:v>
@@ -30370,7 +30398,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O266" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P266" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -30426,7 +30454,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O267" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P267" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -30482,7 +30510,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O268" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P268" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -30538,7 +30566,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O269" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P269" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -30594,7 +30622,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O270" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P270" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -30650,7 +30678,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O271" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P271" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -30706,7 +30734,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O272" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P272" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -30762,7 +30790,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O273" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P273" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -30818,7 +30846,7 @@
         <x:v>配置/Skill/模型/部署版本；provider request ID；环境标识</x:v>
       </x:c>
       <x:c r="O274" s="13" t="str">
-        <x:v>服务health；配置启停；队列queued/processing/DLQ</x:v>
+        <x:v>服务健康状态；配置启停；后台任务状态</x:v>
       </x:c>
       <x:c r="P274" s="13" t="str">
         <x:v>配置缺失、密钥无效、限流、部署失败、队列积压、重复定时任务</x:v>
@@ -31000,58 +31028,58 @@
     </x:row>
     <x:row r="278">
       <x:c r="A278" t="str">
-        <x:v>第 3 期</x:v>
+        <x:v>第 1 期</x:v>
       </x:c>
       <x:c r="B278" t="str">
-        <x:v>6. 平台、工程与上线</x:v>
+        <x:v>2. 图片生成与结果</x:v>
       </x:c>
       <x:c r="C278" t="str">
-        <x:v>INF-DOMAIN-001</x:v>
+        <x:v>GEN-RUNTIME-001</x:v>
       </x:c>
       <x:c r="D278" t="str">
-        <x:v>正式域名</x:v>
+        <x:v>本地真实图片生成链路</x:v>
       </x:c>
       <x:c r="E278" t="str">
-        <x:v>BE-DOMAIN-01</x:v>
+        <x:v>BE-GEN-RUNTIME-01</x:v>
       </x:c>
       <x:c r="F278" t="str">
-        <x:v>后端/基础设施</x:v>
+        <x:v>后端</x:v>
       </x:c>
       <x:c r="G278" t="str">
-        <x:v>注册或确定正式域名</x:v>
+        <x:v>贯通Sub2API、Worker与Supabase真实生成链路</x:v>
       </x:c>
       <x:c r="H278" t="str">
-        <x:v>Bamboo IconGen域名与注册商账号</x:v>
+        <x:v>开发环境本地任务执行器与真实Image 2适配</x:v>
       </x:c>
       <x:c r="I278" t="str">
-        <x:v>域名归项目方控制且可管理DNS</x:v>
+        <x:v>创建任务后本地启动Worker；真实图片逐方案写入Storage；状态可从processing更新为completed并在结果页回显</x:v>
       </x:c>
       <x:c r="J278" t="str">
-        <x:v>—</x:v>
+        <x:v>BE-GEN-STYLE-01</x:v>
       </x:c>
       <x:c r="K278" t="str">
-        <x:v>待完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L278" t="str">
-        <x:v>09-22～09-24</x:v>
+        <x:v>08-25</x:v>
       </x:c>
       <x:c r="M278" t="str">
-        <x:v>—</x:v>
+        <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N278" t="str">
-        <x:v>邮件服务商账号；发信域名；SMTP配置版本；邮箱供应商；测试用户ID</x:v>
+        <x:v>job_id；provider request ID；storage_bucket/path；IMAGE_PROVIDER_BASE_URL</x:v>
       </x:c>
       <x:c r="O278" t="str">
-        <x:v>domain_pending/domain_verified/smtp_pending/smtp_active；邮件sent/delivered/bounced/failed</x:v>
+        <x:v>queued/processing/completed/failed；单图请求成功/失败</x:v>
       </x:c>
       <x:c r="P278" t="str">
-        <x:v>DNS未生效、SMTP鉴权失败、频率限制、邮件进垃圾箱、验证链接过期或回跳失败</x:v>
+        <x:v>Provider限流、图片缺少base64、Storage签名失败、Worker环境缺失</x:v>
       </x:c>
       <x:c r="Q278" t="str">
-        <x:v>SMTP密钥仅服务端保存；日志脱敏；CAPTCHA与速率限制；测试账号最小权限</x:v>
+        <x:v>local-generation-runner.ts；run-job.ts；openai-image-provider.ts；Supabase admin读取与下载路由；Worker/Shared/Web测试和类型检查通过</x:v>
       </x:c>
       <x:c r="R278" t="str">
-        <x:v>团队邮箱先联调；生产SMTP后置；邮件发送和验证操作可重试且不重复赠点</x:v>
+        <x:v>移除AWS/SQS/Lambda依赖；开发环境直接执行Worker；API密钥仅保存在忽略的本地.env</x:v>
       </x:c>
     </x:row>
     <x:row r="279">
@@ -32004,6 +32032,62 @@
       </x:c>
       <x:c r="R295" t="str">
         <x:v>purpose保持可选以兼容旧任务；编译器默认interaction；任务处理可重入</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="296">
+      <x:c r="A296" t="str">
+        <x:v>第 1 期</x:v>
+      </x:c>
+      <x:c r="B296" t="str">
+        <x:v>2. 图片生成与结果</x:v>
+      </x:c>
+      <x:c r="C296" t="str">
+        <x:v>GEN-RUNTIME-001</x:v>
+      </x:c>
+      <x:c r="D296" t="str">
+        <x:v>本地真实图片生成链路</x:v>
+      </x:c>
+      <x:c r="E296" t="str">
+        <x:v>BE-GEN-RUNTIME-01</x:v>
+      </x:c>
+      <x:c r="F296" t="str">
+        <x:v>后端</x:v>
+      </x:c>
+      <x:c r="G296" t="str">
+        <x:v>贯通Sub2API、Worker与Supabase真实生成链路</x:v>
+      </x:c>
+      <x:c r="H296" t="str">
+        <x:v>开发环境本地任务执行器与真实Image 2适配</x:v>
+      </x:c>
+      <x:c r="I296" t="str">
+        <x:v>创建任务后本地启动Worker；真实图片逐方案写入Storage；状态可从processing更新为completed并在结果页回显</x:v>
+      </x:c>
+      <x:c r="J296" t="str">
+        <x:v>BE-GEN-STYLE-01</x:v>
+      </x:c>
+      <x:c r="K296" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="L296" t="str">
+        <x:v>08-25</x:v>
+      </x:c>
+      <x:c r="M296" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N296" t="str">
+        <x:v>job_id；provider request ID；storage_bucket/path；IMAGE_PROVIDER_BASE_URL</x:v>
+      </x:c>
+      <x:c r="O296" t="str">
+        <x:v>queued/processing/completed/failed；单图请求成功/失败</x:v>
+      </x:c>
+      <x:c r="P296" t="str">
+        <x:v>Provider限流、图片缺少base64、Storage签名失败、Worker环境缺失</x:v>
+      </x:c>
+      <x:c r="Q296" t="str">
+        <x:v>local-generation-runner.ts；run-job.ts；openai-image-provider.ts；Supabase admin读取与下载路由；Worker/Shared/Web测试和类型检查通过</x:v>
+      </x:c>
+      <x:c r="R296" t="str">
+        <x:v>移除AWS/SQS/Lambda依赖；开发环境直接执行Worker；API密钥仅保存在忽略的本地.env</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -32022,7 +32106,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R575de5599def4bdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16704f0bb6d34a38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add structured icon style skill and playful preview
</commit_message>
<xml_diff>
--- a/outputs/2026-08-22-style-preview-deployment/IconGen-前后端原子级开发计划.xlsx
+++ b/outputs/2026-08-22-style-preview-deployment/IconGen-前后端原子级开发计划.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段概览" sheetId="1" r:id="Ra90d1b347ca44fad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前端开发计划" sheetId="2" r:id="R1a1c54a083504cd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后端开发计划" sheetId="3" r:id="R166b8c2af78a45b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段概览" sheetId="1" r:id="R384ac5866b034a25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前端开发计划" sheetId="2" r:id="R532ddd5df7f54638"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后端开发计划" sheetId="3" r:id="Re2cc306777ae4962"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -205,7 +205,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FrontendAtomicPlan" displayName="FrontendAtomicPlan" ref="A3:R270" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FrontendAtomicPlan" displayName="FrontendAtomicPlan" ref="A3:R273" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="阶段"/>
     <x:tableColumn id="2" name="大需求/业务模块"/>
@@ -231,7 +231,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BackendAtomicPlan" displayName="BackendAtomicPlan" ref="A3:R278" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BackendAtomicPlan" displayName="BackendAtomicPlan" ref="A3:R281" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="阶段"/>
     <x:tableColumn id="2" name="大需求/业务模块"/>
@@ -475,7 +475,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>更新时间：2026-08-25；完成结果卡片操作精简、终态更新时间隐藏、三方案提示词差异化和原图/高清预览/正式输出三级资产链路；Web、Icon Skill、Worker测试与类型检查通过，真实生成及ZIP链路验收完成</x:v>
+        <x:v>更新时间：2026-08-26；扁平活泼预览资产更新为 v3 并已接入前端；第10个共享预设、9种App图标详细特征规范、Icon Skill 0.5.0 结构化编译器与源图/画布非付费质量告警已完成</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
@@ -515,17 +515,17 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="D4" s="14" t="n">
-        <x:v>256</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="E4" s="14" t="n">
-        <x:v>149</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="F4" s="14" t="n">
         <x:v>107</x:v>
       </x:c>
       <x:c r="G4" s="15" t="n">
         <x:f>E4/D4</x:f>
-        <x:v>0.58203125</x:v>
+        <x:v>0.5868725868725869</x:v>
       </x:c>
       <x:c r="H4" s="14" t="str">
         <x:v>一个动作、一个交付物、一个独立验收结果</x:v>
@@ -542,17 +542,16 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="D5" s="14" t="n">
-        <x:v>274</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="E5" s="14" t="n">
-        <x:v>109</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="F5" s="14" t="n">
         <x:v>165</x:v>
       </x:c>
       <x:c r="G5" s="15" t="n">
-        <x:f>E5/D5</x:f>
-        <x:v>0.3978102189781022</x:v>
+        <x:v>0.4043321299638989</x:v>
       </x:c>
       <x:c r="H5" s="14" t="str">
         <x:v>一个动作、一个交付物、一个独立验收结果</x:v>
@@ -15242,6 +15241,174 @@
       <x:c r="Q270"/>
       <x:c r="R270"/>
     </x:row>
+    <x:row r="271">
+      <x:c r="A271" t="str">
+        <x:v>第 1 期</x:v>
+      </x:c>
+      <x:c r="B271" t="str">
+        <x:v>2. 图片生成与结果</x:v>
+      </x:c>
+      <x:c r="C271" t="str">
+        <x:v>GEN-STYLE-001</x:v>
+      </x:c>
+      <x:c r="D271" t="str">
+        <x:v>App图标风格目录</x:v>
+      </x:c>
+      <x:c r="E271" t="str">
+        <x:v>FE-GEN-STYLE-02</x:v>
+      </x:c>
+      <x:c r="F271" t="str">
+        <x:v>前端</x:v>
+      </x:c>
+      <x:c r="G271" t="str">
+        <x:v>新增扁平活泼风格预设</x:v>
+      </x:c>
+      <x:c r="H271" t="str">
+        <x:v>第10个共享预设、双语文案与高清预览资产</x:v>
+      </x:c>
+      <x:c r="I271" t="str">
+        <x:v>共享目录包含10项；App图标界面展示9项；扁平活泼预览可正常加载</x:v>
+      </x:c>
+      <x:c r="J271" t="str">
+        <x:v>FE-GEN-PREVIEW-03</x:v>
+      </x:c>
+      <x:c r="K271" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="L271" t="str">
+        <x:v>08-25</x:v>
+      </x:c>
+      <x:c r="M271" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N271" t="str">
+        <x:v>preset/settingsVersion/skillVersion；预览资产路径与哈希</x:v>
+      </x:c>
+      <x:c r="O271" t="str">
+        <x:v>目录发布/提示词编译/生成/质量告警</x:v>
+      </x:c>
+      <x:c r="P271" t="str">
+        <x:v>风格漂移、背景边界错误、小尺寸不可读、旧任务兼容</x:v>
+      </x:c>
+      <x:c r="Q271" t="str">
+        <x:v>不包含密钥、用户内容与品牌仿制指令</x:v>
+      </x:c>
+      <x:c r="R271" t="str">
+        <x:v>表格追加可重入；版本号明确；不改变既有任务记录</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="272">
+      <x:c r="A272" t="str">
+        <x:v>第 1 期</x:v>
+      </x:c>
+      <x:c r="B272" t="str">
+        <x:v>2. 图片生成与结果</x:v>
+      </x:c>
+      <x:c r="C272" t="str">
+        <x:v>GEN-STYLE-001</x:v>
+      </x:c>
+      <x:c r="D272" t="str">
+        <x:v>风格契约同步</x:v>
+      </x:c>
+      <x:c r="E272" t="str">
+        <x:v>FE-GEN-STYLE-03</x:v>
+      </x:c>
+      <x:c r="F272" t="str">
+        <x:v>前端</x:v>
+      </x:c>
+      <x:c r="G272" t="str">
+        <x:v>同步风格目录Schema与前端测试</x:v>
+      </x:c>
+      <x:c r="H272" t="str">
+        <x:v>10项目录长度约束与Web契约测试</x:v>
+      </x:c>
+      <x:c r="I272" t="str">
+        <x:v>Shared与Web测试均验证10个预设；线性图标仍仅用于交互图标</x:v>
+      </x:c>
+      <x:c r="J272" t="str">
+        <x:v>FE-GEN-STYLE-02</x:v>
+      </x:c>
+      <x:c r="K272" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="L272" t="str">
+        <x:v>08-25</x:v>
+      </x:c>
+      <x:c r="M272" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N272" t="str">
+        <x:v>preset/settingsVersion/skillVersion；预览资产路径与哈希</x:v>
+      </x:c>
+      <x:c r="O272" t="str">
+        <x:v>目录发布/提示词编译/生成/质量告警</x:v>
+      </x:c>
+      <x:c r="P272" t="str">
+        <x:v>风格漂移、背景边界错误、小尺寸不可读、旧任务兼容</x:v>
+      </x:c>
+      <x:c r="Q272" t="str">
+        <x:v>不包含密钥、用户内容与品牌仿制指令</x:v>
+      </x:c>
+      <x:c r="R272" t="str">
+        <x:v>表格追加可重入；版本号明确；不改变既有任务记录</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="273">
+      <x:c r="A273" t="str">
+        <x:v>第 1 期</x:v>
+      </x:c>
+      <x:c r="B273" t="str">
+        <x:v>2. 图片生成与结果</x:v>
+      </x:c>
+      <x:c r="C273" t="str">
+        <x:v>GEN-STYLE-001</x:v>
+      </x:c>
+      <x:c r="D273" t="str">
+        <x:v>App图标风格目录</x:v>
+      </x:c>
+      <x:c r="E273" t="str">
+        <x:v>FE-GEN-STYLE-04</x:v>
+      </x:c>
+      <x:c r="F273" t="str">
+        <x:v>前端</x:v>
+      </x:c>
+      <x:c r="G273" t="str">
+        <x:v>替换扁平活泼预览资产为 v3</x:v>
+      </x:c>
+      <x:c r="H273" t="str">
+        <x:v>flat-playful-v3.png 与前端目录引用</x:v>
+      </x:c>
+      <x:c r="I273" t="str">
+        <x:v>创建页读取 v3 高清预览；完整原背景无黑底、无展示板且风格细节清晰</x:v>
+      </x:c>
+      <x:c r="J273" t="str">
+        <x:v>FE-GEN-STYLE-03</x:v>
+      </x:c>
+      <x:c r="K273" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="L273" t="str">
+        <x:v>08-26</x:v>
+      </x:c>
+      <x:c r="M273" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
+      <x:c r="N273" t="str">
+        <x:v>preset/settingsVersion/skillVersion；预览资产路径与哈希</x:v>
+      </x:c>
+      <x:c r="O273" t="str">
+        <x:v>目录发布/提示词编译/生成/质量告警</x:v>
+      </x:c>
+      <x:c r="P273" t="str">
+        <x:v>风格漂移、背景边界错误、小尺寸不可读、旧任务兼容</x:v>
+      </x:c>
+      <x:c r="Q273" t="str">
+        <x:v>不包含密钥、用户内容与品牌仿制指令</x:v>
+      </x:c>
+      <x:c r="R273" t="str">
+        <x:v>表格追加可重入；版本号明确；不改变既有任务记录</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:R1"/>
@@ -15258,7 +15425,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9d2b360e6ae4c32"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f20f7bdac7748d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30694,28 +30861,28 @@
         <x:v>2. 图片生成与结果</x:v>
       </x:c>
       <x:c r="C279" t="str">
-        <x:v>GEN-ASSET-001</x:v>
+        <x:v>GEN-PROMPT-001</x:v>
       </x:c>
       <x:c r="D279" t="str">
-        <x:v>高清预览资产</x:v>
+        <x:v>结构化Icon Skill</x:v>
       </x:c>
       <x:c r="E279" t="str">
-        <x:v>BE-GEN-ASSET-01</x:v>
+        <x:v>BE-GEN-PROMPT-02</x:v>
       </x:c>
       <x:c r="F279" t="str">
         <x:v>后端</x:v>
       </x:c>
       <x:c r="G279" t="str">
-        <x:v>建立原图预览图与输出图三级资产</x:v>
+        <x:v>将Icon Skill重构为用途、风格与生产边界编译器</x:v>
       </x:c>
       <x:c r="H279" t="str">
-        <x:v>source、512px preview、requested output资产链路</x:v>
+        <x:v>icon-skill 0.5.0模块化提示词编译器</x:v>
       </x:c>
       <x:c r="I279" t="str">
-        <x:v>结果页使用preview.png；正式下载只使用output；真实任务3方案完成并可ZIP</x:v>
+        <x:v>interaction/app-icon分别应用用途模板；共享边界与三方案方向稳定组合</x:v>
       </x:c>
       <x:c r="J279" t="str">
-        <x:v>BE-GEN-RUNTIME-01</x:v>
+        <x:v>BE-GEN-PROMPT-01</x:v>
       </x:c>
       <x:c r="K279" t="str">
         <x:v>已完成</x:v>
@@ -30727,60 +30894,132 @@
         <x:v>2026-08-25</x:v>
       </x:c>
       <x:c r="N279" t="str">
-        <x:v>asset_role=source/preview/output；preview=512</x:v>
+        <x:v>preset/settingsVersion/skillVersion；预览资产路径与哈希</x:v>
       </x:c>
       <x:c r="O279" t="str">
-        <x:v>处理中/已保存/已完成/失败</x:v>
+        <x:v>目录发布/提示词编译/生成/质量告警</x:v>
       </x:c>
       <x:c r="P279" t="str">
-        <x:v>尺寸约束、预览模糊、资产角色混用</x:v>
+        <x:v>风格漂移、背景边界错误、小尺寸不可读、旧任务兼容</x:v>
       </x:c>
       <x:c r="Q279" t="str">
-        <x:v>私有Bucket、短时签名URL、所有权校验</x:v>
+        <x:v>不包含密钥、用户内容与品牌仿制指令</x:v>
       </x:c>
       <x:c r="R279" t="str">
-        <x:v>迁移0009/0010；Worker测试8项；真实端到端任务完成</x:v>
+        <x:v>表格追加可重入；版本号明确；不改变既有任务记录</x:v>
       </x:c>
     </x:row>
     <x:row r="280">
-      <x:c r="A280"/>
-      <x:c r="B280"/>
-      <x:c r="C280"/>
-      <x:c r="D280"/>
-      <x:c r="E280"/>
-      <x:c r="F280"/>
-      <x:c r="G280"/>
-      <x:c r="H280"/>
-      <x:c r="I280"/>
-      <x:c r="J280"/>
-      <x:c r="K280"/>
-      <x:c r="L280"/>
-      <x:c r="M280"/>
-      <x:c r="N280"/>
-      <x:c r="O280"/>
-      <x:c r="P280"/>
-      <x:c r="Q280"/>
-      <x:c r="R280"/>
+      <x:c r="A280" t="str">
+        <x:v>第 1 期</x:v>
+      </x:c>
+      <x:c r="B280" t="str">
+        <x:v>2. 图片生成与结果</x:v>
+      </x:c>
+      <x:c r="C280" t="str">
+        <x:v>GEN-PROMPT-001</x:v>
+      </x:c>
+      <x:c r="D280" t="str">
+        <x:v>详细风格规范</x:v>
+      </x:c>
+      <x:c r="E280" t="str">
+        <x:v>BE-GEN-PROMPT-03</x:v>
+      </x:c>
+      <x:c r="F280" t="str">
+        <x:v>后端</x:v>
+      </x:c>
+      <x:c r="G280" t="str">
+        <x:v>为9种App图标风格建立详细特征规范</x:v>
+      </x:c>
+      <x:c r="H280" t="str">
+        <x:v>9份独立风格spec</x:v>
+      </x:c>
+      <x:c r="I280" t="str">
+        <x:v>每种风格均包含构图、配色或材质、光影或层次、边缘细节及小尺寸规则</x:v>
+      </x:c>
+      <x:c r="J280" t="str">
+        <x:v>BE-GEN-PROMPT-02</x:v>
+      </x:c>
+      <x:c r="K280" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="L280" t="str">
+        <x:v>08-25</x:v>
+      </x:c>
+      <x:c r="M280" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N280" t="str">
+        <x:v>preset/settingsVersion/skillVersion；预览资产路径与哈希</x:v>
+      </x:c>
+      <x:c r="O280" t="str">
+        <x:v>目录发布/提示词编译/生成/质量告警</x:v>
+      </x:c>
+      <x:c r="P280" t="str">
+        <x:v>风格漂移、背景边界错误、小尺寸不可读、旧任务兼容</x:v>
+      </x:c>
+      <x:c r="Q280" t="str">
+        <x:v>不包含密钥、用户内容与品牌仿制指令</x:v>
+      </x:c>
+      <x:c r="R280" t="str">
+        <x:v>表格追加可重入；版本号明确；不改变既有任务记录</x:v>
+      </x:c>
     </x:row>
     <x:row r="281">
-      <x:c r="A281"/>
-      <x:c r="B281"/>
-      <x:c r="C281"/>
-      <x:c r="D281"/>
-      <x:c r="E281"/>
-      <x:c r="F281"/>
-      <x:c r="G281"/>
-      <x:c r="H281"/>
-      <x:c r="I281"/>
-      <x:c r="J281"/>
-      <x:c r="K281"/>
-      <x:c r="L281"/>
-      <x:c r="M281"/>
-      <x:c r="N281"/>
-      <x:c r="O281"/>
-      <x:c r="P281"/>
-      <x:c r="Q281"/>
-      <x:c r="R281"/>
+      <x:c r="A281" t="str">
+        <x:v>第 1 期</x:v>
+      </x:c>
+      <x:c r="B281" t="str">
+        <x:v>2. 图片生成与结果</x:v>
+      </x:c>
+      <x:c r="C281" t="str">
+        <x:v>GEN-QUALITY-001</x:v>
+      </x:c>
+      <x:c r="D281" t="str">
+        <x:v>生成图片质量门</x:v>
+      </x:c>
+      <x:c r="E281" t="str">
+        <x:v>BE-GEN-QUALITY-01</x:v>
+      </x:c>
+      <x:c r="F281" t="str">
+        <x:v>后端</x:v>
+      </x:c>
+      <x:c r="G281" t="str">
+        <x:v>增加非付费源图与画布质量检查</x:v>
+      </x:c>
+      <x:c r="H281" t="str">
+        <x:v>SharpImageQualityGate及单元测试</x:v>
+      </x:c>
+      <x:c r="I281" t="str">
+        <x:v>检测低于1024、非正方形和App图标深色外角；仅记录结构化告警不重复计费</x:v>
+      </x:c>
+      <x:c r="J281" t="str">
+        <x:v>BE-GEN-PROMPT-02</x:v>
+      </x:c>
+      <x:c r="K281" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="L281" t="str">
+        <x:v>08-25</x:v>
+      </x:c>
+      <x:c r="M281" t="str">
+        <x:v>2026-08-25</x:v>
+      </x:c>
+      <x:c r="N281" t="str">
+        <x:v>preset/settingsVersion/skillVersion；预览资产路径与哈希</x:v>
+      </x:c>
+      <x:c r="O281" t="str">
+        <x:v>目录发布/提示词编译/生成/质量告警</x:v>
+      </x:c>
+      <x:c r="P281" t="str">
+        <x:v>风格漂移、背景边界错误、小尺寸不可读、旧任务兼容</x:v>
+      </x:c>
+      <x:c r="Q281" t="str">
+        <x:v>不包含密钥、用户内容与品牌仿制指令</x:v>
+      </x:c>
+      <x:c r="R281" t="str">
+        <x:v>表格追加可重入；版本号明确；不改变既有任务记录</x:v>
+      </x:c>
     </x:row>
     <x:row r="282">
       <x:c r="A282"/>
@@ -31098,7 +31337,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R542d77ea138d40a6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5df9571931194187"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: harden icon generation quality workflow
</commit_message>
<xml_diff>
--- a/outputs/2026-08-22-style-preview-deployment/IconGen-前后端原子级开发计划.xlsx
+++ b/outputs/2026-08-22-style-preview-deployment/IconGen-前后端原子级开发计划.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段概览" sheetId="1" r:id="R384ac5866b034a25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前端开发计划" sheetId="2" r:id="R532ddd5df7f54638"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后端开发计划" sheetId="3" r:id="Re2cc306777ae4962"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段概览" sheetId="1" r:id="R51fa15eff8ae42ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前端开发计划" sheetId="2" r:id="R4409587bf1e24e68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后端开发计划" sheetId="3" r:id="R6410eea32193449d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -231,7 +231,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BackendAtomicPlan" displayName="BackendAtomicPlan" ref="A3:R281" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BackendAtomicPlan" displayName="BackendAtomicPlan" ref="A3:R284" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="18">
     <x:tableColumn id="1" name="阶段"/>
     <x:tableColumn id="2" name="大需求/业务模块"/>
@@ -475,7 +475,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>更新时间：2026-08-26；扁平活泼预览资产更新为 v3 并已接入前端；第10个共享预设、9种App图标详细特征规范、Icon Skill 0.5.0 结构化编译器与源图/画布非付费质量告警已完成</x:v>
+        <x:v>更新时间：2026-08-30；Icon Skill 0.8.8 已完成分风格质量契约、Image2 不透明/透明背景参数、定向质量重试与失败终态诊断；九种 App 图标风格真实回归 27/27 方案完成</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
@@ -542,16 +542,17 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="D5" s="14" t="n">
-        <x:v>277</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="E5" s="14" t="n">
-        <x:v>112</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="F5" s="14" t="n">
         <x:v>165</x:v>
       </x:c>
       <x:c r="G5" s="15" t="n">
-        <x:v>0.4043321299638989</x:v>
+        <x:f>E5/D5</x:f>
+        <x:v>0.4107142857142857</x:v>
       </x:c>
       <x:c r="H5" s="14" t="str">
         <x:v>一个动作、一个交付物、一个独立验收结果</x:v>
@@ -15425,7 +15426,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f20f7bdac7748d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R650c6502db644090"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31022,64 +31023,172 @@
       </x:c>
     </x:row>
     <x:row r="282">
-      <x:c r="A282"/>
-      <x:c r="B282"/>
-      <x:c r="C282"/>
-      <x:c r="D282"/>
-      <x:c r="E282"/>
-      <x:c r="F282"/>
-      <x:c r="G282"/>
-      <x:c r="H282"/>
-      <x:c r="I282"/>
-      <x:c r="J282"/>
-      <x:c r="K282"/>
-      <x:c r="L282"/>
-      <x:c r="M282"/>
-      <x:c r="N282"/>
-      <x:c r="O282"/>
-      <x:c r="P282"/>
-      <x:c r="Q282"/>
-      <x:c r="R282"/>
+      <x:c r="A282" t="str">
+        <x:v>第 1 期</x:v>
+      </x:c>
+      <x:c r="B282" t="str">
+        <x:v>2. 图片生成与结果</x:v>
+      </x:c>
+      <x:c r="C282" t="str">
+        <x:v>GEN-QUALITY-001</x:v>
+      </x:c>
+      <x:c r="D282" t="str">
+        <x:v>分风格质量门与终态</x:v>
+      </x:c>
+      <x:c r="E282" t="str">
+        <x:v>BE-GEN-QUALITY-02</x:v>
+      </x:c>
+      <x:c r="F282" t="str">
+        <x:v>后端</x:v>
+      </x:c>
+      <x:c r="G282" t="str">
+        <x:v>实现分风格背景质量契约与方案失败终态</x:v>
+      </x:c>
+      <x:c r="H282" t="str">
+        <x:v>Icon Skill 0.8.7 qualityContract、边缘连通检测与失败诊断</x:v>
+      </x:c>
+      <x:c r="I282" t="str">
+        <x:v>不同风格使用独立质量阈值；失败方案立即进入failed；任务终态不遗留queued或processing</x:v>
+      </x:c>
+      <x:c r="J282" t="str">
+        <x:v>BE-GEN-QUALITY-01</x:v>
+      </x:c>
+      <x:c r="K282" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="L282" t="str">
+        <x:v>08-30</x:v>
+      </x:c>
+      <x:c r="M282" t="str">
+        <x:v>2026-08-30</x:v>
+      </x:c>
+      <x:c r="N282" t="str">
+        <x:v>style preset；quality profile；border/canvas coverage；target color distance；variant status</x:v>
+      </x:c>
+      <x:c r="O282" t="str">
+        <x:v>queued/processing/completed/failed；job completed/partial/failed</x:v>
+      </x:c>
+      <x:c r="P282" t="str">
+        <x:v>统一阈值误报、黑边漏检、任务终态覆盖方案诊断、方案状态卡死</x:v>
+      </x:c>
+      <x:c r="Q282" t="str">
+        <x:v>服务端仅记录质量指标；错误消息截断；不输出Provider或Supabase密钥</x:v>
+      </x:c>
+      <x:c r="R282" t="str">
+        <x:v>8项Skill测试、25项Worker测试和四工作区类型检查通过；真实任务无终态状态残留</x:v>
+      </x:c>
     </x:row>
     <x:row r="283">
-      <x:c r="A283"/>
-      <x:c r="B283"/>
-      <x:c r="C283"/>
-      <x:c r="D283"/>
-      <x:c r="E283"/>
-      <x:c r="F283"/>
-      <x:c r="G283"/>
-      <x:c r="H283"/>
-      <x:c r="I283"/>
-      <x:c r="J283"/>
-      <x:c r="K283"/>
-      <x:c r="L283"/>
-      <x:c r="M283"/>
-      <x:c r="N283"/>
-      <x:c r="O283"/>
-      <x:c r="P283"/>
-      <x:c r="Q283"/>
-      <x:c r="R283"/>
+      <x:c r="A283" t="str">
+        <x:v>第 1 期</x:v>
+      </x:c>
+      <x:c r="B283" t="str">
+        <x:v>2. 图片生成与结果</x:v>
+      </x:c>
+      <x:c r="C283" t="str">
+        <x:v>GEN-QUALITY-001</x:v>
+      </x:c>
+      <x:c r="D283" t="str">
+        <x:v>Image2背景与定向重试</x:v>
+      </x:c>
+      <x:c r="E283" t="str">
+        <x:v>BE-GEN-QUALITY-03</x:v>
+      </x:c>
+      <x:c r="F283" t="str">
+        <x:v>后端</x:v>
+      </x:c>
+      <x:c r="G283" t="str">
+        <x:v>向Image2传递背景模式并根据质量诊断重试</x:v>
+      </x:c>
+      <x:c r="H283" t="str">
+        <x:v>Icon Skill 0.8.8、opaque/transparent参数与MANDATORY RETRY REPAIR提示</x:v>
+      </x:c>
+      <x:c r="I283" t="str">
+        <x:v>有背景任务传opaque；透明任务传transparent；后续尝试包含上一轮具体质量问题且重新渲染</x:v>
+      </x:c>
+      <x:c r="J283" t="str">
+        <x:v>BE-GEN-QUALITY-02</x:v>
+      </x:c>
+      <x:c r="K283" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="L283" t="str">
+        <x:v>08-30</x:v>
+      </x:c>
+      <x:c r="M283" t="str">
+        <x:v>2026-08-30</x:v>
+      </x:c>
+      <x:c r="N283" t="str">
+        <x:v>outputBackground；quality warning code/message；quality attempt；provider request ID</x:v>
+      </x:c>
+      <x:c r="O283" t="str">
+        <x:v>首次生成/质量拒绝/定向重试/完成/失败</x:v>
+      </x:c>
+      <x:c r="P283" t="str">
+        <x:v>网关不支持参数、重复同一缺陷、无背景描述与质量契约冲突、霓虹暗角误报</x:v>
+      </x:c>
+      <x:c r="Q283" t="str">
+        <x:v>不记录API密钥；仅向既有Image2网关发送生成参数与任务提示词</x:v>
+      </x:c>
+      <x:c r="R283" t="str">
+        <x:v>新增参数与重试单测；修复无背景契约冲突；霓虹跳过无效暗角告警</x:v>
+      </x:c>
     </x:row>
     <x:row r="284">
-      <x:c r="A284"/>
-      <x:c r="B284"/>
-      <x:c r="C284"/>
-      <x:c r="D284"/>
-      <x:c r="E284"/>
-      <x:c r="F284"/>
-      <x:c r="G284"/>
-      <x:c r="H284"/>
-      <x:c r="I284"/>
-      <x:c r="J284"/>
-      <x:c r="K284"/>
-      <x:c r="L284"/>
-      <x:c r="M284"/>
-      <x:c r="N284"/>
-      <x:c r="O284"/>
-      <x:c r="P284"/>
-      <x:c r="Q284"/>
-      <x:c r="R284"/>
+      <x:c r="A284" t="str">
+        <x:v>第 1 期</x:v>
+      </x:c>
+      <x:c r="B284" t="str">
+        <x:v>2. 图片生成与结果</x:v>
+      </x:c>
+      <x:c r="C284" t="str">
+        <x:v>GEN-QA-001</x:v>
+      </x:c>
+      <x:c r="D284" t="str">
+        <x:v>九风格真实链路回归</x:v>
+      </x:c>
+      <x:c r="E284" t="str">
+        <x:v>BE-GEN-QA-01</x:v>
+      </x:c>
+      <x:c r="F284" t="str">
+        <x:v>后端/测试</x:v>
+      </x:c>
+      <x:c r="G284" t="str">
+        <x:v>执行九种App图标风格真实Image2回归</x:v>
+      </x:c>
+      <x:c r="H284" t="str">
+        <x:v>9个随机用户案例、27个真实方案及任务ID记录</x:v>
+      </x:c>
+      <x:c r="I284" t="str">
+        <x:v>黏土3D、等距3D、低多边形、霓虹、像素艺术、扁平插画、扁平活泼、可爱贴纸、极简标志均3/3 completed</x:v>
+      </x:c>
+      <x:c r="J284" t="str">
+        <x:v>BE-GEN-QUALITY-03</x:v>
+      </x:c>
+      <x:c r="K284" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="L284" t="str">
+        <x:v>08-30</x:v>
+      </x:c>
+      <x:c r="M284" t="str">
+        <x:v>2026-08-30</x:v>
+      </x:c>
+      <x:c r="N284" t="str">
+        <x:v>job ID；preset；variant status；quality warning；skillVersion=0.8.8</x:v>
+      </x:c>
+      <x:c r="O284" t="str">
+        <x:v>queued/processing/completed/partial/failed</x:v>
+      </x:c>
+      <x:c r="P284" t="str">
+        <x:v>限流、黑角、白边、背景不均匀、质量门误报、终态残留</x:v>
+      </x:c>
+      <x:c r="Q284" t="str">
+        <x:v>测试使用现有私有配置；记录中不保存密钥；任务仅属于当前测试用户</x:v>
+      </x:c>
+      <x:c r="R284" t="str">
+        <x:v>9个任务全部completed；27/27方案完成；无failed、partial、queued或processing残留</x:v>
+      </x:c>
     </x:row>
     <x:row r="285">
       <x:c r="A285"/>
@@ -31337,7 +31446,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5df9571931194187"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5abd8c56eb2048d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: harden icon generation backgrounds and runtime
</commit_message>
<xml_diff>
--- a/outputs/2026-08-22-style-preview-deployment/IconGen-前后端原子级开发计划.xlsx
+++ b/outputs/2026-08-22-style-preview-deployment/IconGen-前后端原子级开发计划.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段概览" sheetId="1" r:id="R51fa15eff8ae42ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前端开发计划" sheetId="2" r:id="R4409587bf1e24e68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后端开发计划" sheetId="3" r:id="R6410eea32193449d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段概览" sheetId="1" r:id="R55bd308ee0754f03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="前端开发计划" sheetId="2" r:id="R2e0159f3ce994b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="后端开发计划" sheetId="3" r:id="R70380ec52e064d95"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -475,7 +475,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>更新时间：2026-08-30；Icon Skill 0.8.8 已完成分风格质量契约、Image2 不透明/透明背景参数、定向质量重试与失败终态诊断；九种 App 图标风格真实回归 27/27 方案完成</x:v>
+        <x:v>更新时间：2026-09-01；已完成 App 插画图标逐主体背景形状/圆角角度设置与真实 Image2 回归：14% 圆角任务 3/3 方案完成并写入 Supabase Storage；Sub2API 图像账号已绑定 image-2 分组。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
@@ -15410,6 +15410,62 @@
         <x:v>表格追加可重入；版本号明确；不改变既有任务记录</x:v>
       </x:c>
     </x:row>
+    <x:row r="274">
+      <x:c r="A274" t="str">
+        <x:v>第 1 期</x:v>
+      </x:c>
+      <x:c r="B274" t="str">
+        <x:v>2. 图片生成与结果</x:v>
+      </x:c>
+      <x:c r="C274" t="str">
+        <x:v>GEN-APP-BACKGROUND-001</x:v>
+      </x:c>
+      <x:c r="D274" t="str">
+        <x:v>App 插画图标背景</x:v>
+      </x:c>
+      <x:c r="E274" t="str">
+        <x:v>FE-GEN-APP-BG-01</x:v>
+      </x:c>
+      <x:c r="F274" t="str">
+        <x:v>前端</x:v>
+      </x:c>
+      <x:c r="G274" t="str">
+        <x:v>支持逐主体设置背景形状与圆角角度</x:v>
+      </x:c>
+      <x:c r="H274" t="str">
+        <x:v>主体草稿背景模式、形状与 4%–40% 圆角控件</x:v>
+      </x:c>
+      <x:c r="I274" t="str">
+        <x:v>切换 App 插画图标后每个主体均展示独立背景设置；Rounded 状态支持滑动与数值输入；提交值写入对应主体背景覆盖</x:v>
+      </x:c>
+      <x:c r="J274" t="str">
+        <x:v>FE-GEN-SUBJECT-01</x:v>
+      </x:c>
+      <x:c r="K274" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="L274" t="str">
+        <x:v>09-01</x:v>
+      </x:c>
+      <x:c r="M274" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="N274" t="str">
+        <x:v>subject.backgroundOverride.cornerRadius；container；purpose=app-icon</x:v>
+      </x:c>
+      <x:c r="O274" t="str">
+        <x:v>透明/单色/渐变；rounded/circle/square；4%–40%</x:v>
+      </x:c>
+      <x:c r="P274" t="str">
+        <x:v>用途切换丢失设置、数值越界、主体间串值、旧草稿缺值</x:v>
+      </x:c>
+      <x:c r="Q274" t="str">
+        <x:v>不采集用户敏感数据；仅提交生成规格</x:v>
+      </x:c>
+      <x:c r="R274" t="str">
+        <x:v>generation-subject-drafts.ts；AppIconBackgroundSettings；generation-form；Reducer/Web测试、typecheck、lint通过；14%真实任务参数已写入数据库</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:R1"/>
@@ -15426,7 +15482,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R650c6502db644090"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4140f393e5134c17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31191,24 +31247,60 @@
       </x:c>
     </x:row>
     <x:row r="285">
-      <x:c r="A285"/>
-      <x:c r="B285"/>
-      <x:c r="C285"/>
-      <x:c r="D285"/>
-      <x:c r="E285"/>
-      <x:c r="F285"/>
-      <x:c r="G285"/>
-      <x:c r="H285"/>
-      <x:c r="I285"/>
-      <x:c r="J285"/>
-      <x:c r="K285"/>
-      <x:c r="L285"/>
-      <x:c r="M285"/>
-      <x:c r="N285"/>
-      <x:c r="O285"/>
-      <x:c r="P285"/>
-      <x:c r="Q285"/>
-      <x:c r="R285"/>
+      <x:c r="A285" t="str">
+        <x:v>第 1 期</x:v>
+      </x:c>
+      <x:c r="B285" t="str">
+        <x:v>2. 图片生成与结果</x:v>
+      </x:c>
+      <x:c r="C285" t="str">
+        <x:v>GEN-RUNTIME-002</x:v>
+      </x:c>
+      <x:c r="D285" t="str">
+        <x:v>Image2 图像账号调度与圆角真实回归</x:v>
+      </x:c>
+      <x:c r="E285" t="str">
+        <x:v>BE-GEN-RUNTIME-02</x:v>
+      </x:c>
+      <x:c r="F285" t="str">
+        <x:v>后端/测试</x:v>
+      </x:c>
+      <x:c r="G285" t="str">
+        <x:v>修复 Sub2API 图像账号分组并验证逐主体圆角生成链路</x:v>
+      </x:c>
+      <x:c r="H285" t="str">
+        <x:v>image-2 分组账号绑定、真实 Image2 任务与 Storage 母版</x:v>
+      </x:c>
+      <x:c r="I285" t="str">
+        <x:v>gpt-image-2 最小请求成功；14% rounded-square 背景任务 3 个方案全部 completed；每个 1254px 原图均带 Alpha 并写入 Storage</x:v>
+      </x:c>
+      <x:c r="J285" t="str">
+        <x:v>BE-GEN-RUNTIME-01</x:v>
+      </x:c>
+      <x:c r="K285" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="L285" t="str">
+        <x:v>09-01</x:v>
+      </x:c>
+      <x:c r="M285" t="str">
+        <x:v>2026-09-01</x:v>
+      </x:c>
+      <x:c r="N285" t="str">
+        <x:v>IMAGE_MODEL；Sub2API group；backgroundOverride.cornerRadius；provider request ID；asset path</x:v>
+      </x:c>
+      <x:c r="O285" t="str">
+        <x:v>Sub2API 账号未分组/已分组；queued/processing/completed</x:v>
+      </x:c>
+      <x:c r="P285" t="str">
+        <x:v>模型可列出但无可调度账号、503、网关与Worker配置不一致、圆角掩码未写入资产</x:v>
+      </x:c>
+      <x:c r="Q285" t="str">
+        <x:v>不记录网关密钥；仅管理员管理账号分组；生成请求仅含任务提示词</x:v>
+      </x:c>
+      <x:c r="R285" t="str">
+        <x:v>管理员将唯一 OpenAI OAuth 账号加入 image-2 分组；最小 gpt-image-2 调用成功；真实任务 eb3f22f9-6c8f-479b-98bd-1c0f6fa69581 3/3 completed</x:v>
+      </x:c>
     </x:row>
     <x:row r="286">
       <x:c r="A286"/>
@@ -31446,7 +31538,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5abd8c56eb2048d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c7615487dc14f35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>